<commit_message>
feat: incrementando tela para seleção de arquivos, visualização de resultados e alterando o metodo de comparação
</commit_message>
<xml_diff>
--- a/analise.xlsx
+++ b/analise.xlsx
@@ -18,10 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -60,12 +57,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,16 +468,20 @@
           <t>039.173.221-88</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>19993</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1954-09-26</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>70297</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>70297</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -495,62 +495,74 @@
           <t>876.995.634-09</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>33689</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1992-03-26</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>69314</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>69314</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yasmin Eliane Agatha Gonçalves</t>
+          <t>Marina Sophie Marlene da Luz</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>193.703.911-00</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>16635</v>
+          <t>369.960.476-41</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1944-02-05</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>61902</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38045</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marina Sophie Marlene da Luz</t>
+          <t>Yasmin Eliane Agatha Gonçalves</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>369.960.476-41</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>16107</v>
+          <t>193.703.911-00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1945-07-17</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>38045</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>61902</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -564,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,31 +605,6 @@
           <t>Matricula</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>chaveCPF&amp;Nome</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>chaveCPF&amp;DtNasc</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>chaveCPF&amp;Sexo</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>chaveCPF&amp;Matricula</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>chave</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -630,40 +617,19 @@
           <t>876.995.634-09</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>33689</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1992-03-26</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>69314</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>876.995.634-09Anthony Henrique Costa</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>876.995.634-091992-03-26</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>876.995.634-09M</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>876.995.634-0969314</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>876.995.634-09Anthony Henrique Costa1992-03-26M69314</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>69314</t>
         </is>
       </c>
     </row>
@@ -678,40 +644,19 @@
           <t>039.173.221-88</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>19993</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1954-09-26</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>70297</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>039.173.221-88Mário Manoel Calebe Moura</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>039.173.221-881954-09-26</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>039.173.221-88M</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>039.173.221-8870297</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>039.173.221-88Mário Manoel Calebe Moura1954-09-26M70297</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>70297</t>
         </is>
       </c>
     </row>
@@ -726,40 +671,19 @@
           <t>193.703.911-00</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>16635</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1945-07-17</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>61902</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>193.703.911-00Yasmin Eliane Agatha Gonçalves</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>193.703.911-001945-07-17</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>193.703.911-00F</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>193.703.911-0061902</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>193.703.911-00Yasmin Eliane Agatha Gonçalves1945-07-17F61902</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>61902</t>
         </is>
       </c>
     </row>
@@ -774,40 +698,19 @@
           <t>369.960.476-41</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>16107</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1944-02-05</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>38045</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>369.960.476-41Marina Sophie Marlene da Luz</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>369.960.476-411944-02-05</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>369.960.476-41F</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>369.960.476-4138045</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>369.960.476-41Marina Sophie Marlene da Luz1944-02-05F38045</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>38045</t>
         </is>
       </c>
     </row>
@@ -822,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -858,50 +761,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>chaveCPF&amp;Nome</t>
+          <t>ComparaCPF_Nome</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>ComparaCPF_Nome</t>
+          <t>ComparaCPF_DtNasc</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>chaveCPF&amp;DtNasc</t>
+          <t>ComparaCPF_Sexo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ComparaCPF_DtNasc</t>
+          <t>ComparaCPF_Matricula</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>chaveCPF&amp;Sexo</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>ComparaCPF_Sexo</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>chaveCPF&amp;Matricula</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>ComparaCPF_Matricula</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>chave</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
@@ -918,16 +796,20 @@
           <t>039.173.221-88</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>19993</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1954-09-26</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>70297</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>70297</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -936,7 +818,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>039.173.221-88Mário Manoel Calebe Moura</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -946,7 +828,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>039.173.221-881954-09-26</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -955,31 +837,6 @@
         </is>
       </c>
       <c r="K2" t="inlineStr">
-        <is>
-          <t>039.173.221-88M</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>039.173.221-8870297</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>039.173.221-88Mário Manoel Calebe Moura1954-09-26M70297</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
         <is>
           <t>Localizado</t>
         </is>
@@ -996,16 +853,20 @@
           <t>876.995.634-09</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>33689</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1992-03-26</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>69314</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>69314</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1014,7 +875,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>876.995.634-09Anthony Henrique Costa</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1024,7 +885,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>876.995.634-091992-03-26</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1033,31 +894,6 @@
         </is>
       </c>
       <c r="K3" t="inlineStr">
-        <is>
-          <t>876.995.634-09M</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>876.995.634-0969314</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>876.995.634-09Anthony Henrique Costa1992-03-26M69314</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
         <is>
           <t>Localizado</t>
         </is>
@@ -1066,24 +902,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yasmin Eliane Agatha Gonçalves</t>
+          <t>Marina Sophie Marlene da Luz</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>193.703.911-00</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>16635</v>
+          <t>369.960.476-41</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1944-02-05</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>61902</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38045</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1092,7 +932,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>193.703.911-00Yasmin Eliane Agatha Gonçalves</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1102,7 +942,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>193.703.911-001945-07-17</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1111,31 +951,6 @@
         </is>
       </c>
       <c r="K4" t="inlineStr">
-        <is>
-          <t>193.703.911-00F</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>193.703.911-0061902</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>193.703.911-00Yasmin Eliane Agatha Gonçalves1945-07-17F61902</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
         <is>
           <t>Localizado</t>
         </is>
@@ -1144,24 +959,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marina Sophie Marlene da Luz</t>
+          <t>Yasmin Eliane Agatha Gonçalves</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>369.960.476-41</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>16107</v>
+          <t>193.703.911-00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1945-07-17</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>38045</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>61902</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1170,7 +989,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>369.960.476-41Marina Sophie Marlene da Luz</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1180,7 +999,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>369.960.476-411944-02-05</t>
+          <t>Localizado</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1189,31 +1008,6 @@
         </is>
       </c>
       <c r="K5" t="inlineStr">
-        <is>
-          <t>369.960.476-41F</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>369.960.476-4138045</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Localizado</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>369.960.476-41Marina Sophie Marlene da Luz1944-02-05F38045</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
         <is>
           <t>Localizado</t>
         </is>

</xml_diff>